<commit_message>
added sliding window questions
</commit_message>
<xml_diff>
--- a/DSA Sheet - Trishansh.xlsx
+++ b/DSA Sheet - Trishansh.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA SHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBF936B-3D13-467E-B9C4-8DA61B5B61C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64CD9C78-8399-488B-907D-AF796D9728B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Binary Search" sheetId="1" r:id="rId1"/>
     <sheet name="Array Searching and Rotation" sheetId="3" r:id="rId2"/>
     <sheet name="Two Pointer - Array" sheetId="4" r:id="rId3"/>
+    <sheet name="Sliding Window" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
   <si>
     <t xml:space="preserve">Question </t>
   </si>
@@ -129,6 +130,18 @@
   </si>
   <si>
     <t xml:space="preserve">  Revision(April)</t>
+  </si>
+  <si>
+    <t>Maximum Sum Subarray of size k</t>
+  </si>
+  <si>
+    <t>Sliding Window (Array) Practice Questions</t>
+  </si>
+  <si>
+    <t>Minimum Sum Subarray of size k</t>
+  </si>
+  <si>
+    <t>Longest Subarray with sum &lt;= k</t>
   </si>
 </sst>
 </file>
@@ -847,4 +860,74 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{951F55F9-E1D5-4BCD-A88A-1212BAF00F8F}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="37" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="90.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.77734375" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="5"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="5"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="1"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add Strings practice questions
</commit_message>
<xml_diff>
--- a/DSA Sheet - Trishansh.xlsx
+++ b/DSA Sheet - Trishansh.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA SHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D051957-907B-4598-8821-C2810DD9BA33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F732F7C0-D189-48F4-87E0-23C83E812632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Binary Search" sheetId="1" r:id="rId1"/>
-    <sheet name="Array Searching and Rotation" sheetId="3" r:id="rId2"/>
-    <sheet name="Two Pointer - Array" sheetId="4" r:id="rId3"/>
-    <sheet name="Sliding Window" sheetId="5" r:id="rId4"/>
-    <sheet name="Stack" sheetId="6" r:id="rId5"/>
+    <sheet name="Strings" sheetId="7" r:id="rId2"/>
+    <sheet name="Array Searching and Rotation" sheetId="3" r:id="rId3"/>
+    <sheet name="Two Pointer - Array" sheetId="4" r:id="rId4"/>
+    <sheet name="Sliding Window" sheetId="5" r:id="rId5"/>
+    <sheet name="Stack" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="52">
   <si>
     <t xml:space="preserve">Question </t>
   </si>
@@ -158,6 +159,33 @@
   </si>
   <si>
     <t>Remove consecutive duplicates from string</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strings Practice Questions </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reverse a String </t>
+  </si>
+  <si>
+    <t>Reverse words in a sentence</t>
+  </si>
+  <si>
+    <t>Reverse characters of a string</t>
+  </si>
+  <si>
+    <t>Check if a string is Palindrome</t>
+  </si>
+  <si>
+    <t>Check if two strings are anagrams</t>
+  </si>
+  <si>
+    <t>Check Substring</t>
+  </si>
+  <si>
+    <t>Character frequency count</t>
+  </si>
+  <si>
+    <t>Remove duplicates from a string</t>
   </si>
 </sst>
 </file>
@@ -189,7 +217,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -211,6 +239,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -243,7 +283,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
@@ -252,6 +292,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -651,6 +693,104 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A586BF35-5C97-4FD8-ABCB-13C9B2E56421}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="44.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="6"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="6"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="6"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="6"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="6"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="6"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="6"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="6"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63803EBD-65BB-4CB1-86D0-A17F7488F714}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -764,7 +904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24AFF5C3-4FB1-4FCA-A387-86E3D53367A5}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -878,7 +1018,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{951F55F9-E1D5-4BCD-A88A-1212BAF00F8F}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -948,7 +1088,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8FC88D9-D983-4DA5-B5B8-E5B51188E6E7}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
added more strings questions
</commit_message>
<xml_diff>
--- a/DSA Sheet - Trishansh.xlsx
+++ b/DSA Sheet - Trishansh.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA SHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F732F7C0-D189-48F4-87E0-23C83E812632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B9C18D2-D82C-4ABE-8303-10398A863520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="53">
   <si>
     <t xml:space="preserve">Question </t>
   </si>
@@ -186,6 +186,9 @@
   </si>
   <si>
     <t>Remove duplicates from a string</t>
+  </si>
+  <si>
+    <t>Run-length encoding of a string(compress consecuitve chars)</t>
   </si>
 </sst>
 </file>
@@ -697,7 +700,7 @@
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="44.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="84.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -781,9 +784,11 @@
       <c r="C11" s="6"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="1"/>
+      <c r="A12" s="7" t="s">
+        <v>52</v>
+      </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="C12" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added more strings practice questions
</commit_message>
<xml_diff>
--- a/DSA Sheet - Trishansh.xlsx
+++ b/DSA Sheet - Trishansh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA SHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B9C18D2-D82C-4ABE-8303-10398A863520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1AEF05-5131-49C4-926E-650ED0E95CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="56">
   <si>
     <t xml:space="preserve">Question </t>
   </si>
@@ -189,6 +189,15 @@
   </si>
   <si>
     <t>Run-length encoding of a string(compress consecuitve chars)</t>
+  </si>
+  <si>
+    <t>Find first non-repeating characters in a string</t>
+  </si>
+  <si>
+    <t>Check if two strings can be made equal by swapping two chars</t>
+  </si>
+  <si>
+    <t>Longest common prefix among array of strings</t>
   </si>
 </sst>
 </file>
@@ -697,10 +706,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A586BF35-5C97-4FD8-ABCB-13C9B2E56421}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="52.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="54.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="84.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -789,6 +798,52 @@
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="6"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="6"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="6"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="6"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added binary search questions
</commit_message>
<xml_diff>
--- a/DSA Sheet - Trishansh.xlsx
+++ b/DSA Sheet - Trishansh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA SHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1AEF05-5131-49C4-926E-650ED0E95CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30FB3D0B-FD29-4374-9037-A05D19AEB154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="60">
   <si>
     <t xml:space="preserve">Question </t>
   </si>
@@ -198,6 +198,18 @@
   </si>
   <si>
     <t>Longest common prefix among array of strings</t>
+  </si>
+  <si>
+    <t>Check if a string is rotation of another</t>
+  </si>
+  <si>
+    <t>Count occurences of a pattern in a string(naive search)</t>
+  </si>
+  <si>
+    <t>Find longest palindromic substring</t>
+  </si>
+  <si>
+    <t>Roman numeral to integer</t>
   </si>
 </sst>
 </file>
@@ -821,24 +833,32 @@
       <c r="C15" s="6"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
+      <c r="A16" s="7" t="s">
+        <v>56</v>
+      </c>
       <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+      <c r="C16" s="6"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
+      <c r="A17" s="7" t="s">
+        <v>57</v>
+      </c>
       <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+      <c r="C17" s="6"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
+      <c r="A18" s="7" t="s">
+        <v>58</v>
+      </c>
       <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
+      <c r="C18" s="6"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
+      <c r="A19" s="7" t="s">
+        <v>59</v>
+      </c>
       <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
+      <c r="C19" s="6"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>

</xml_diff>

<commit_message>
added more searching questions
</commit_message>
<xml_diff>
--- a/DSA Sheet - Trishansh.xlsx
+++ b/DSA Sheet - Trishansh.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA SHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30FB3D0B-FD29-4374-9037-A05D19AEB154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E2C39A-8D97-429C-A393-A29ED1DD97FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Binary Search" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="62">
   <si>
     <t xml:space="preserve">Question </t>
   </si>
@@ -41,9 +41,6 @@
     <t>https://leetcode.com/problems/binary-search/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Binary Search </t>
-  </si>
-  <si>
     <t>Find first and last position of element in sorted array</t>
   </si>
   <si>
@@ -210,6 +207,15 @@
   </si>
   <si>
     <t>Roman numeral to integer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary Search ( Iterative ) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary Search ( Recursive ) </t>
+  </si>
+  <si>
+    <t>Count occurences of element in sorted array</t>
   </si>
 </sst>
 </file>
@@ -599,17 +605,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="44.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="84.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1"/>
     </row>
@@ -626,12 +632,12 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
+      <c r="A4" s="7" t="s">
+        <v>59</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>2</v>
@@ -639,78 +645,92 @@
       <c r="C4" s="3"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="A7" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="2"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="3"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId1" xr:uid="{B0554624-DA0B-4CD4-9FA9-CD9380540178}"/>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{B0554624-DA0B-4CD4-9FA9-CD9380540178}"/>
     <hyperlink ref="B4" r:id="rId2" xr:uid="{A45BC86A-8696-482F-8F0E-55EC484FD42A}"/>
-    <hyperlink ref="B6" r:id="rId3" xr:uid="{2FD665CD-3828-4755-9611-FCFF9D500D40}"/>
-    <hyperlink ref="B7" r:id="rId4" xr:uid="{C25A050B-ACC4-4F41-8870-C793DD927CC9}"/>
-    <hyperlink ref="B8" r:id="rId5" xr:uid="{CAD8D048-F9AA-4ACD-8562-7FCE30D08109}"/>
-    <hyperlink ref="B9" r:id="rId6" xr:uid="{ADCDD71B-CBBC-4A93-B87B-0E032FE683E1}"/>
-    <hyperlink ref="B10" r:id="rId7" xr:uid="{14BBEED7-187F-48BF-B092-A3C877C3AF4C}"/>
+    <hyperlink ref="B8" r:id="rId3" xr:uid="{2FD665CD-3828-4755-9611-FCFF9D500D40}"/>
+    <hyperlink ref="B9" r:id="rId4" xr:uid="{C25A050B-ACC4-4F41-8870-C793DD927CC9}"/>
+    <hyperlink ref="B10" r:id="rId5" xr:uid="{CAD8D048-F9AA-4ACD-8562-7FCE30D08109}"/>
+    <hyperlink ref="B11" r:id="rId6" xr:uid="{ADCDD71B-CBBC-4A93-B87B-0E032FE683E1}"/>
+    <hyperlink ref="B12" r:id="rId7" xr:uid="{14BBEED7-187F-48BF-B092-A3C877C3AF4C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -728,7 +748,7 @@
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1"/>
     </row>
@@ -745,117 +765,117 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="6"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="6"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="6"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="6"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="6"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="6"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="6"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="6"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="6"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="6"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="6"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="6"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="6"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="6"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="6"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="6"/>
@@ -883,7 +903,7 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -902,25 +922,25 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>2</v>
@@ -930,17 +950,17 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="3"/>
@@ -997,7 +1017,7 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C1" s="1"/>
     </row>
@@ -1014,48 +1034,48 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -1112,7 +1132,7 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1"/>
     </row>
@@ -1129,13 +1149,13 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="3"/>
@@ -1143,7 +1163,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="3"/>
@@ -1151,7 +1171,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="3"/>
@@ -1182,7 +1202,7 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C1" s="1"/>
     </row>
@@ -1199,13 +1219,13 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="3"/>
@@ -1213,7 +1233,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="3"/>
@@ -1221,7 +1241,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="3"/>
@@ -1229,7 +1249,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="3"/>

</xml_diff>

<commit_message>
solved Merge Intervals question
</commit_message>
<xml_diff>
--- a/DSA Sheet - Trishansh.xlsx
+++ b/DSA Sheet - Trishansh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA SHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B91B33-2FDE-4BDA-8416-E4B385C1226B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7381E3A3-8D32-4689-A1BB-A35072142813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
   <si>
     <t xml:space="preserve">Question </t>
   </si>
@@ -253,6 +253,9 @@
   </si>
   <si>
     <t>Find median of two sorted arrays</t>
+  </si>
+  <si>
+    <t>Merge Intervals (sort by start, then merge overlapping)</t>
   </si>
 </sst>
 </file>
@@ -788,7 +791,7 @@
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.5546875" customWidth="1"/>
+    <col min="1" max="1" width="49.77734375" customWidth="1"/>
     <col min="2" max="2" width="90.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.109375" customWidth="1"/>
   </cols>
@@ -875,11 +878,11 @@
       <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>69</v>
+      <c r="A12" s="7" t="s">
+        <v>74</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="C12" s="3"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B16" t="s">

</xml_diff>

<commit_message>
Practiced 2D Arrays questions
</commit_message>
<xml_diff>
--- a/DSA Sheet - Trishansh.xlsx
+++ b/DSA Sheet - Trishansh.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA SHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7381E3A3-8D32-4689-A1BB-A35072142813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4979BF2-8199-4493-A2F8-51FC83D408D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Binary Search" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,8 @@
     <sheet name="Array Searching and Rotation" sheetId="3" r:id="rId4"/>
     <sheet name="Two Pointer - Array" sheetId="4" r:id="rId5"/>
     <sheet name="Sliding Window" sheetId="5" r:id="rId6"/>
-    <sheet name="Stack" sheetId="6" r:id="rId7"/>
+    <sheet name="2D Arrays " sheetId="9" r:id="rId7"/>
+    <sheet name="Stack" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="85">
   <si>
     <t xml:space="preserve">Question </t>
   </si>
@@ -256,6 +257,36 @@
   </si>
   <si>
     <t>Merge Intervals (sort by start, then merge overlapping)</t>
+  </si>
+  <si>
+    <t>2D Arrays Practice Questions</t>
+  </si>
+  <si>
+    <t>Print Matrix row and column wise</t>
+  </si>
+  <si>
+    <t>Print Main Diagonal and Secondary Diagonal</t>
+  </si>
+  <si>
+    <t>Search Element in Matrix (Linear Search)</t>
+  </si>
+  <si>
+    <t>Search Element in Sorted Matrix (Binary Search)</t>
+  </si>
+  <si>
+    <t>Count Even and Odd numbers in matrix</t>
+  </si>
+  <si>
+    <t>Find Maximum element in matrix</t>
+  </si>
+  <si>
+    <t>Sum of each row , Sum of each column</t>
+  </si>
+  <si>
+    <t>Row with Maximum Sum</t>
+  </si>
+  <si>
+    <t>Transpose of Matrix</t>
   </si>
 </sst>
 </file>
@@ -1347,6 +1378,165 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{488613D1-50CD-4BCD-9774-E05D95780B47}">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="47.77734375" customWidth="1"/>
+    <col min="2" max="2" width="47.33203125" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="5"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="5"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="1"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="1"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8FC88D9-D983-4DA5-B5B8-E5B51188E6E7}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Solved 2D arrays advance questions
</commit_message>
<xml_diff>
--- a/DSA Sheet - Trishansh.xlsx
+++ b/DSA Sheet - Trishansh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA SHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4979BF2-8199-4493-A2F8-51FC83D408D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ABEF25F-B966-4249-A22C-5BE0305DDAF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="91">
   <si>
     <t xml:space="preserve">Question </t>
   </si>
@@ -287,6 +287,24 @@
   </si>
   <si>
     <t>Transpose of Matrix</t>
+  </si>
+  <si>
+    <t>Transpose of Matrix (in place) Square Matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rotate matrix by 180 degrees </t>
+  </si>
+  <si>
+    <t>Rotate matrix by 90 degrees (Clock-wise)</t>
+  </si>
+  <si>
+    <t>Zig-Zag Traversal</t>
+  </si>
+  <si>
+    <t>Wave Traversal (Column-wise)</t>
+  </si>
+  <si>
+    <t>Matrix Multiplication</t>
   </si>
 </sst>
 </file>
@@ -1484,39 +1502,51 @@
       <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
+      <c r="A13" s="1" t="s">
+        <v>85</v>
+      </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="C13" s="3"/>
       <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
+      <c r="A14" s="1" t="s">
+        <v>87</v>
+      </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+      <c r="C14" s="3"/>
       <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
+      <c r="A15" s="1" t="s">
+        <v>86</v>
+      </c>
       <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+      <c r="C15" s="3"/>
       <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
+      <c r="A16" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+      <c r="C16" s="3"/>
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
+      <c r="A17" s="1" t="s">
+        <v>89</v>
+      </c>
       <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+      <c r="C17" s="3"/>
       <c r="D17" s="1"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
+      <c r="A18" s="1" t="s">
+        <v>90</v>
+      </c>
       <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
+      <c r="C18" s="3"/>
       <c r="D18" s="1"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>